<commit_message>
use of if condition and different formulas in worksheet
</commit_message>
<xml_diff>
--- a/EXCEL/Details.xlsx
+++ b/EXCEL/Details.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dhane\Videos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/898af4500e89e0da/Desktop/DHRUV/Data Science and Analytics with GenAl/EXCEL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A6152608-415B-42DB-98F4-35F8CA028FB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="8_{A6152608-415B-42DB-98F4-35F8CA028FB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{04454F36-2DE9-4DB9-BA1A-85B0404501C8}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{5C010742-0D1E-4B81-84DF-4C0EBDAA81F1}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{5C010742-0D1E-4B81-84DF-4C0EBDAA81F1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="42">
   <si>
     <t>ID</t>
   </si>
@@ -159,6 +159,9 @@
   </si>
   <si>
     <t>Tanya Bedi</t>
+  </si>
+  <si>
+    <t>high/low</t>
   </si>
 </sst>
 </file>
@@ -550,10 +553,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CFD4C5C-D03E-4B7A-A44B-431478AFBB18}">
-  <dimension ref="A1:J21"/>
-  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:K21"/>
+  <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.4"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -584,8 +587,11 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" ht="42" x14ac:dyDescent="0.35">
+      <c r="K1" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="42" x14ac:dyDescent="0.4">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -616,8 +622,12 @@
       <c r="J2" s="2">
         <v>135000</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" ht="42" x14ac:dyDescent="0.35">
+      <c r="K2" t="str">
+        <f>IF(E2&gt;29, "high", "low")</f>
+        <v>low</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="42" x14ac:dyDescent="0.4">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -648,8 +658,12 @@
       <c r="J3" s="2">
         <v>104000</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" ht="42" x14ac:dyDescent="0.35">
+      <c r="K3" t="str">
+        <f t="shared" ref="K3:K4" si="0">IF(E3&gt;29, "high", "low")</f>
+        <v>low</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -680,8 +694,12 @@
       <c r="J4" s="2">
         <v>150000</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" ht="42" x14ac:dyDescent="0.35">
+      <c r="K4" t="str">
+        <f t="shared" si="0"/>
+        <v>high</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -712,8 +730,12 @@
       <c r="J5" s="2">
         <v>98000</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" ht="42" x14ac:dyDescent="0.35">
+      <c r="K5" t="str">
+        <f t="shared" ref="K3:K21" si="1">IF(E5&gt;29, "high", "low")</f>
+        <v>low</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="42" x14ac:dyDescent="0.4">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -744,8 +766,12 @@
       <c r="J6" s="2">
         <v>97000</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" ht="42" x14ac:dyDescent="0.35">
+      <c r="K6" t="str">
+        <f t="shared" si="1"/>
+        <v>low</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="42" x14ac:dyDescent="0.4">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -776,8 +802,12 @@
       <c r="J7" s="2">
         <v>82000</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" ht="42" x14ac:dyDescent="0.35">
+      <c r="K7" t="str">
+        <f t="shared" si="1"/>
+        <v>high</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="42" x14ac:dyDescent="0.4">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -808,8 +838,12 @@
       <c r="J8" s="2">
         <v>140000</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K8" t="str">
+        <f t="shared" si="1"/>
+        <v>high</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -840,8 +874,12 @@
       <c r="J9" s="2">
         <v>96000</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" ht="42" x14ac:dyDescent="0.35">
+      <c r="K9" t="str">
+        <f t="shared" si="1"/>
+        <v>low</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -872,8 +910,12 @@
       <c r="J10" s="2">
         <v>112000</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" ht="42" x14ac:dyDescent="0.35">
+      <c r="K10" t="str">
+        <f t="shared" si="1"/>
+        <v>high</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="42" x14ac:dyDescent="0.4">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -904,8 +946,12 @@
       <c r="J11" s="2">
         <v>103000</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K11" t="str">
+        <f t="shared" si="1"/>
+        <v>high</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -936,8 +982,12 @@
       <c r="J12" s="2">
         <v>136000</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" ht="42" x14ac:dyDescent="0.35">
+      <c r="K12" t="str">
+        <f t="shared" si="1"/>
+        <v>low</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -968,8 +1018,12 @@
       <c r="J13" s="2">
         <v>92000</v>
       </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K13" t="str">
+        <f t="shared" si="1"/>
+        <v>low</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -1000,8 +1054,12 @@
       <c r="J14" s="2">
         <v>101000</v>
       </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K14" t="str">
+        <f t="shared" si="1"/>
+        <v>high</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -1032,8 +1090,12 @@
       <c r="J15" s="2">
         <v>90000</v>
       </c>
-    </row>
-    <row r="16" spans="1:10" ht="42" x14ac:dyDescent="0.35">
+      <c r="K15" t="str">
+        <f t="shared" si="1"/>
+        <v>low</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="42" x14ac:dyDescent="0.4">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -1064,8 +1126,12 @@
       <c r="J16" s="2">
         <v>123000</v>
       </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K16" t="str">
+        <f t="shared" si="1"/>
+        <v>high</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -1096,8 +1162,12 @@
       <c r="J17" s="2">
         <v>142000</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" ht="42" x14ac:dyDescent="0.35">
+      <c r="K17" t="str">
+        <f t="shared" si="1"/>
+        <v>low</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="42" x14ac:dyDescent="0.4">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -1128,8 +1198,12 @@
       <c r="J18" s="2">
         <v>100000</v>
       </c>
-    </row>
-    <row r="19" spans="1:10" ht="42" x14ac:dyDescent="0.35">
+      <c r="K18" t="str">
+        <f t="shared" si="1"/>
+        <v>low</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="42" x14ac:dyDescent="0.4">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -1160,8 +1234,12 @@
       <c r="J19" s="2">
         <v>91000</v>
       </c>
-    </row>
-    <row r="20" spans="1:10" ht="42" x14ac:dyDescent="0.35">
+      <c r="K19" t="str">
+        <f t="shared" si="1"/>
+        <v>low</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="42" x14ac:dyDescent="0.4">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -1192,8 +1270,12 @@
       <c r="J20" s="2">
         <v>128000</v>
       </c>
-    </row>
-    <row r="21" spans="1:10" ht="42" x14ac:dyDescent="0.35">
+      <c r="K20" t="str">
+        <f t="shared" si="1"/>
+        <v>high</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -1223,6 +1305,10 @@
       </c>
       <c r="J21" s="2">
         <v>137000</v>
+      </c>
+      <c r="K21" t="str">
+        <f t="shared" si="1"/>
+        <v>high</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
use of and, or operator in excel sheet
</commit_message>
<xml_diff>
--- a/EXCEL/Details.xlsx
+++ b/EXCEL/Details.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/898af4500e89e0da/Desktop/DHRUV/Data Science and Analytics with GenAl/EXCEL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="8_{A6152608-415B-42DB-98F4-35F8CA028FB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{04454F36-2DE9-4DB9-BA1A-85B0404501C8}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="8_{A6152608-415B-42DB-98F4-35F8CA028FB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF1DBFBB-2AF7-48DC-BAA5-5455075BB366}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{5C010742-0D1E-4B81-84DF-4C0EBDAA81F1}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="43">
   <si>
     <t>ID</t>
   </si>
@@ -162,6 +162,9 @@
   </si>
   <si>
     <t>high/low</t>
+  </si>
+  <si>
+    <t>and/or</t>
   </si>
 </sst>
 </file>
@@ -205,11 +208,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -218,6 +218,12 @@
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -234,6 +240,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -553,762 +563,845 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CFD4C5C-D03E-4B7A-A44B-431478AFBB18}">
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.4"/>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="5" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" ht="42" x14ac:dyDescent="0.4">
-      <c r="A2" s="2">
+      <c r="L1" s="5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" ht="42" x14ac:dyDescent="0.4">
+      <c r="A2" s="1">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2" s="2">
         <v>44562</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>28</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="2">
+      <c r="G2" s="1">
         <v>42000</v>
       </c>
-      <c r="H2" s="4">
+      <c r="H2" s="3">
         <v>0.05</v>
       </c>
-      <c r="I2" s="2">
+      <c r="I2" s="1">
         <v>120000</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>135000</v>
       </c>
       <c r="K2" t="str">
         <f>IF(E2&gt;29, "high", "low")</f>
         <v>low</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" ht="42" x14ac:dyDescent="0.4">
-      <c r="A3" s="2">
+      <c r="L2" t="b">
+        <f>AND(G6&gt;50000,I2&gt;10000)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="42" x14ac:dyDescent="0.4">
+      <c r="A3" s="1">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="2">
         <v>44242</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>25</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G3" s="2">
+      <c r="G3" s="1">
         <v>55000</v>
       </c>
-      <c r="H3" s="4">
+      <c r="H3" s="3">
         <v>0.08</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="1">
         <v>98000</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>104000</v>
       </c>
       <c r="K3" t="str">
         <f t="shared" ref="K3:K4" si="0">IF(E3&gt;29, "high", "low")</f>
         <v>low</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A4" s="2">
+      <c r="L3" t="b">
+        <f t="shared" ref="L3:L21" si="1">AND(G7&gt;50000,I3&gt;10000)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="A4" s="1">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="2">
         <v>43910</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>32</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="G4" s="2">
+      <c r="G4" s="1">
         <v>60000</v>
       </c>
-      <c r="H4" s="4">
+      <c r="H4" s="3">
         <v>0.1</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="1">
         <v>145000</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>150000</v>
       </c>
       <c r="K4" t="str">
         <f t="shared" si="0"/>
         <v>high</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A5" s="2">
+      <c r="L4" t="b">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="A5" s="1">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="2">
         <v>45026</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>26</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="F5" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G5" s="2">
+      <c r="G5" s="1">
         <v>38000</v>
       </c>
-      <c r="H5" s="4">
+      <c r="H5" s="3">
         <v>0.06</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="1">
         <v>110000</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>98000</v>
       </c>
       <c r="K5" t="str">
-        <f t="shared" ref="K3:K21" si="1">IF(E5&gt;29, "high", "low")</f>
+        <f t="shared" ref="K5:K21" si="2">IF(E5&gt;29, "high", "low")</f>
         <v>low</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" ht="42" x14ac:dyDescent="0.4">
-      <c r="A6" s="2">
+      <c r="L5" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="42" x14ac:dyDescent="0.4">
+      <c r="A6" s="1">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="2">
         <v>43590</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>29</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F6" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="G6" s="2">
+      <c r="G6" s="1">
         <v>48000</v>
       </c>
-      <c r="H6" s="4">
+      <c r="H6" s="3">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="1">
         <v>89000</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>97000</v>
       </c>
       <c r="K6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>low</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" ht="42" x14ac:dyDescent="0.4">
-      <c r="A7" s="2">
+      <c r="L6" t="b">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="42" x14ac:dyDescent="0.4">
+      <c r="A7" s="1">
         <v>6</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D7" s="2">
         <v>44377</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>31</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F7" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="G7" s="2">
+      <c r="G7" s="1">
         <v>45000</v>
       </c>
-      <c r="H7" s="4">
+      <c r="H7" s="3">
         <v>0.05</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="1">
         <v>77000</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>82000</v>
       </c>
       <c r="K7" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>high</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" ht="42" x14ac:dyDescent="0.4">
-      <c r="A8" s="2">
+      <c r="L7" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="42" x14ac:dyDescent="0.4">
+      <c r="A8" s="1">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D8" s="2">
         <v>44764</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>34</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="G8" s="2">
+      <c r="G8" s="1">
         <v>62000</v>
       </c>
-      <c r="H8" s="4">
+      <c r="H8" s="3">
         <v>0.09</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="1">
         <v>132000</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>140000</v>
       </c>
       <c r="K8" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>high</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A9" s="2">
+      <c r="L8" t="b">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="A9" s="1">
         <v>8</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D9" s="2">
         <v>44054</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>27</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="F9" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="G9" s="2">
+      <c r="G9" s="1">
         <v>39000</v>
       </c>
-      <c r="H9" s="4">
+      <c r="H9" s="3">
         <v>0.06</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="1">
         <v>91000</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>96000</v>
       </c>
       <c r="K9" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>low</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A10" s="2">
+      <c r="L9" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="A10" s="1">
         <v>9</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="3">
+      <c r="D10" s="2">
         <v>44456</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>30</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="F10" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G10" s="2">
+      <c r="G10" s="1">
         <v>52000</v>
       </c>
-      <c r="H10" s="4">
+      <c r="H10" s="3">
         <v>0.08</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="1">
         <v>105000</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>112000</v>
       </c>
       <c r="K10" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>high</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" ht="42" x14ac:dyDescent="0.4">
-      <c r="A11" s="2">
+      <c r="L10" t="b">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="42" x14ac:dyDescent="0.4">
+      <c r="A11" s="1">
         <v>10</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D11" s="3">
+      <c r="D11" s="2">
         <v>43739</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>35</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="F11" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="G11" s="2">
+      <c r="G11" s="1">
         <v>47000</v>
       </c>
-      <c r="H11" s="4">
+      <c r="H11" s="3">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I11" s="1">
         <v>99000</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>103000</v>
       </c>
       <c r="K11" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>high</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A12" s="2">
+      <c r="L11" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="A12" s="1">
         <v>11</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="3">
+      <c r="D12" s="2">
         <v>44149</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>28</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="F12" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G12" s="2">
+      <c r="G12" s="1">
         <v>61000</v>
       </c>
-      <c r="H12" s="4">
+      <c r="H12" s="3">
         <v>0.1</v>
       </c>
-      <c r="I12" s="2">
+      <c r="I12" s="1">
         <v>128000</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>136000</v>
       </c>
       <c r="K12" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>low</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A13" s="2">
+      <c r="L12" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="A13" s="1">
         <v>12</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D13" s="3">
+      <c r="D13" s="2">
         <v>44914</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>24</v>
       </c>
-      <c r="F13" s="2" t="s">
+      <c r="F13" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="G13" s="2">
+      <c r="G13" s="1">
         <v>36000</v>
       </c>
-      <c r="H13" s="4">
+      <c r="H13" s="3">
         <v>0.05</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I13" s="1">
         <v>88000</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>92000</v>
       </c>
       <c r="K13" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>low</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A14" s="2">
+      <c r="L13" t="b">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="A14" s="1">
         <v>13</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D14" s="3">
+      <c r="D14" s="2">
         <v>44204</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>33</v>
       </c>
-      <c r="F14" s="2" t="s">
+      <c r="F14" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="G14" s="2">
+      <c r="G14" s="1">
         <v>54000</v>
       </c>
-      <c r="H14" s="4">
+      <c r="H14" s="3">
         <v>0.09</v>
       </c>
-      <c r="I14" s="2">
+      <c r="I14" s="1">
         <v>97000</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>101000</v>
       </c>
       <c r="K14" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>high</v>
       </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A15" s="2">
+      <c r="L14" t="b">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="A15" s="1">
         <v>14</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C15" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D15" s="3">
+      <c r="D15" s="2">
         <v>43864</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>29</v>
       </c>
-      <c r="F15" s="2" t="s">
+      <c r="F15" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="G15" s="2">
+      <c r="G15" s="1">
         <v>44000</v>
       </c>
-      <c r="H15" s="4">
+      <c r="H15" s="3">
         <v>0.06</v>
       </c>
-      <c r="I15" s="2">
+      <c r="I15" s="1">
         <v>86000</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>90000</v>
       </c>
       <c r="K15" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>low</v>
       </c>
-    </row>
-    <row r="16" spans="1:11" ht="42" x14ac:dyDescent="0.4">
-      <c r="A16" s="2">
+      <c r="L15" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" ht="42" x14ac:dyDescent="0.4">
+      <c r="A16" s="1">
         <v>15</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D16" s="3">
+      <c r="D16" s="2">
         <v>43545</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>31</v>
       </c>
-      <c r="F16" s="2" t="s">
+      <c r="F16" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="G16" s="2">
+      <c r="G16" s="1">
         <v>40000</v>
       </c>
-      <c r="H16" s="4">
+      <c r="H16" s="3">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="I16" s="2">
+      <c r="I16" s="1">
         <v>119000</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>123000</v>
       </c>
       <c r="K16" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>high</v>
       </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A17" s="2">
+      <c r="L16" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="A17" s="1">
         <v>16</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C17" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D17" s="3">
+      <c r="D17" s="2">
         <v>44663</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <v>27</v>
       </c>
-      <c r="F17" s="2" t="s">
+      <c r="F17" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G17" s="2">
+      <c r="G17" s="1">
         <v>59000</v>
       </c>
-      <c r="H17" s="4">
+      <c r="H17" s="3">
         <v>0.1</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17" s="1">
         <v>138000</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>142000</v>
       </c>
       <c r="K17" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>low</v>
       </c>
-    </row>
-    <row r="18" spans="1:11" ht="42" x14ac:dyDescent="0.4">
-      <c r="A18" s="2">
+      <c r="L17" t="b">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" ht="42" x14ac:dyDescent="0.4">
+      <c r="A18" s="1">
         <v>17</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="C18" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D18" s="3">
+      <c r="D18" s="2">
         <v>44345</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>26</v>
       </c>
-      <c r="F18" s="2" t="s">
+      <c r="F18" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G18" s="2">
+      <c r="G18" s="1">
         <v>53000</v>
       </c>
-      <c r="H18" s="4">
+      <c r="H18" s="3">
         <v>0.08</v>
       </c>
-      <c r="I18" s="2">
+      <c r="I18" s="1">
         <v>94000</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>100000</v>
       </c>
       <c r="K18" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>low</v>
       </c>
-    </row>
-    <row r="19" spans="1:11" ht="42" x14ac:dyDescent="0.4">
-      <c r="A19" s="2">
+      <c r="L18" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" ht="42" x14ac:dyDescent="0.4">
+      <c r="A19" s="1">
         <v>18</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="C19" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D19" s="3">
+      <c r="D19" s="2">
         <v>45083</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" s="1">
         <v>25</v>
       </c>
-      <c r="F19" s="2" t="s">
+      <c r="F19" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="G19" s="2">
+      <c r="G19" s="1">
         <v>46000</v>
       </c>
-      <c r="H19" s="4">
+      <c r="H19" s="3">
         <v>0.06</v>
       </c>
-      <c r="I19" s="2">
+      <c r="I19" s="1">
         <v>87000</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>91000</v>
       </c>
       <c r="K19" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>low</v>
       </c>
-    </row>
-    <row r="20" spans="1:11" ht="42" x14ac:dyDescent="0.4">
-      <c r="A20" s="2">
+      <c r="L19" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" ht="42" x14ac:dyDescent="0.4">
+      <c r="A20" s="1">
         <v>19</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C20" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D20" s="3">
+      <c r="D20" s="2">
         <v>43673</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>32</v>
       </c>
-      <c r="F20" s="2" t="s">
+      <c r="F20" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="G20" s="2">
+      <c r="G20" s="1">
         <v>41000</v>
       </c>
-      <c r="H20" s="4">
+      <c r="H20" s="3">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="I20" s="2">
+      <c r="I20" s="1">
         <v>122000</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>128000</v>
       </c>
       <c r="K20" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>high</v>
       </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A21" s="2">
+      <c r="L20" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="A21" s="1">
         <v>20</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C21" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D21" s="3">
+      <c r="D21" s="2">
         <v>44788</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>30</v>
       </c>
-      <c r="F21" s="2" t="s">
+      <c r="F21" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="G21" s="2">
+      <c r="G21" s="1">
         <v>58000</v>
       </c>
-      <c r="H21" s="4">
+      <c r="H21" s="3">
         <v>0.09</v>
       </c>
-      <c r="I21" s="2">
+      <c r="I21" s="1">
         <v>130000</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>137000</v>
       </c>
       <c r="K21" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>high</v>
+      </c>
+      <c r="L21" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
use of not operator in the excel sheet
</commit_message>
<xml_diff>
--- a/EXCEL/Details.xlsx
+++ b/EXCEL/Details.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/898af4500e89e0da/Desktop/DHRUV/Data Science and Analytics with GenAl/EXCEL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="23" documentId="8_{A6152608-415B-42DB-98F4-35F8CA028FB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF1DBFBB-2AF7-48DC-BAA5-5455075BB366}"/>
+  <xr:revisionPtr revIDLastSave="28" documentId="8_{A6152608-415B-42DB-98F4-35F8CA028FB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D0E619BB-F5E3-44DD-9582-1116F9B9D094}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{5C010742-0D1E-4B81-84DF-4C0EBDAA81F1}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="44">
   <si>
     <t>ID</t>
   </si>
@@ -165,6 +165,9 @@
   </si>
   <si>
     <t>and/or</t>
+  </si>
+  <si>
+    <t>not</t>
   </si>
 </sst>
 </file>
@@ -563,10 +566,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CFD4C5C-D03E-4B7A-A44B-431478AFBB18}">
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:M21"/>
   <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.4"/>
   <sheetData>
-    <row r="1" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -603,8 +606,11 @@
       <c r="L1" s="5" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" ht="42" x14ac:dyDescent="0.4">
+      <c r="M1" s="5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="42" x14ac:dyDescent="0.4">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -643,8 +649,12 @@
         <f>AND(G6&gt;50000,I2&gt;10000)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" ht="42" x14ac:dyDescent="0.4">
+      <c r="M2" t="str">
+        <f>IF(NOT(C2="HR"),"OTHER DEPT","HR")</f>
+        <v>HR</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" ht="42" x14ac:dyDescent="0.4">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -683,8 +693,12 @@
         <f t="shared" ref="L3:L21" si="1">AND(G7&gt;50000,I3&gt;10000)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="M3" t="str">
+        <f t="shared" ref="M3:M21" si="2">IF(NOT(C3="HR"),"OTHER DEPT","HR")</f>
+        <v>OTHER DEPT</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -723,8 +737,12 @@
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="M4" t="str">
+        <f t="shared" si="2"/>
+        <v>OTHER DEPT</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -756,15 +774,19 @@
         <v>98000</v>
       </c>
       <c r="K5" t="str">
-        <f t="shared" ref="K5:K21" si="2">IF(E5&gt;29, "high", "low")</f>
+        <f t="shared" ref="K5:K21" si="3">IF(E5&gt;29, "high", "low")</f>
         <v>low</v>
       </c>
       <c r="L5" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" ht="42" x14ac:dyDescent="0.4">
+      <c r="M5" t="str">
+        <f t="shared" si="2"/>
+        <v>OTHER DEPT</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="42" x14ac:dyDescent="0.4">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -796,15 +818,19 @@
         <v>97000</v>
       </c>
       <c r="K6" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>low</v>
       </c>
       <c r="L6" t="b">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:12" ht="42" x14ac:dyDescent="0.4">
+      <c r="M6" t="str">
+        <f t="shared" si="2"/>
+        <v>OTHER DEPT</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" ht="42" x14ac:dyDescent="0.4">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -836,15 +862,19 @@
         <v>82000</v>
       </c>
       <c r="K7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>high</v>
       </c>
       <c r="L7" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:12" ht="42" x14ac:dyDescent="0.4">
+      <c r="M7" t="str">
+        <f t="shared" si="2"/>
+        <v>HR</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" ht="42" x14ac:dyDescent="0.4">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -876,15 +906,19 @@
         <v>140000</v>
       </c>
       <c r="K8" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>high</v>
       </c>
       <c r="L8" t="b">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="M8" t="str">
+        <f t="shared" si="2"/>
+        <v>OTHER DEPT</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -916,15 +950,19 @@
         <v>96000</v>
       </c>
       <c r="K9" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>low</v>
       </c>
       <c r="L9" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="M9" t="str">
+        <f t="shared" si="2"/>
+        <v>OTHER DEPT</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -956,15 +994,19 @@
         <v>112000</v>
       </c>
       <c r="K10" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>high</v>
       </c>
       <c r="L10" t="b">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:12" ht="42" x14ac:dyDescent="0.4">
+      <c r="M10" t="str">
+        <f t="shared" si="2"/>
+        <v>OTHER DEPT</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" ht="42" x14ac:dyDescent="0.4">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -996,15 +1038,19 @@
         <v>103000</v>
       </c>
       <c r="K11" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>high</v>
       </c>
       <c r="L11" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="M11" t="str">
+        <f t="shared" si="2"/>
+        <v>HR</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -1036,15 +1082,19 @@
         <v>136000</v>
       </c>
       <c r="K12" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>low</v>
       </c>
       <c r="L12" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="M12" t="str">
+        <f t="shared" si="2"/>
+        <v>OTHER DEPT</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -1076,15 +1126,19 @@
         <v>92000</v>
       </c>
       <c r="K13" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>low</v>
       </c>
       <c r="L13" t="b">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="M13" t="str">
+        <f t="shared" si="2"/>
+        <v>OTHER DEPT</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -1116,15 +1170,19 @@
         <v>101000</v>
       </c>
       <c r="K14" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>high</v>
       </c>
       <c r="L14" t="b">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="M14" t="str">
+        <f t="shared" si="2"/>
+        <v>OTHER DEPT</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -1156,15 +1214,19 @@
         <v>90000</v>
       </c>
       <c r="K15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>low</v>
       </c>
       <c r="L15" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:12" ht="42" x14ac:dyDescent="0.4">
+      <c r="M15" t="str">
+        <f t="shared" si="2"/>
+        <v>HR</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" ht="42" x14ac:dyDescent="0.4">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -1196,15 +1258,19 @@
         <v>123000</v>
       </c>
       <c r="K16" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>high</v>
       </c>
       <c r="L16" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="M16" t="str">
+        <f t="shared" si="2"/>
+        <v>OTHER DEPT</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A17" s="1">
         <v>16</v>
       </c>
@@ -1236,15 +1302,19 @@
         <v>142000</v>
       </c>
       <c r="K17" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>low</v>
       </c>
       <c r="L17" t="b">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-    </row>
-    <row r="18" spans="1:12" ht="42" x14ac:dyDescent="0.4">
+      <c r="M17" t="str">
+        <f t="shared" si="2"/>
+        <v>OTHER DEPT</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" ht="42" x14ac:dyDescent="0.4">
       <c r="A18" s="1">
         <v>17</v>
       </c>
@@ -1276,15 +1346,19 @@
         <v>100000</v>
       </c>
       <c r="K18" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>low</v>
       </c>
       <c r="L18" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:12" ht="42" x14ac:dyDescent="0.4">
+      <c r="M18" t="str">
+        <f t="shared" si="2"/>
+        <v>OTHER DEPT</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" ht="42" x14ac:dyDescent="0.4">
       <c r="A19" s="1">
         <v>18</v>
       </c>
@@ -1316,15 +1390,19 @@
         <v>91000</v>
       </c>
       <c r="K19" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>low</v>
       </c>
       <c r="L19" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="20" spans="1:12" ht="42" x14ac:dyDescent="0.4">
+      <c r="M19" t="str">
+        <f t="shared" si="2"/>
+        <v>HR</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" ht="42" x14ac:dyDescent="0.4">
       <c r="A20" s="1">
         <v>19</v>
       </c>
@@ -1356,15 +1434,19 @@
         <v>128000</v>
       </c>
       <c r="K20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>high</v>
       </c>
       <c r="L20" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.4">
+      <c r="M20" t="str">
+        <f t="shared" si="2"/>
+        <v>OTHER DEPT</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A21" s="1">
         <v>20</v>
       </c>
@@ -1396,12 +1478,16 @@
         <v>137000</v>
       </c>
       <c r="K21" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>high</v>
       </c>
       <c r="L21" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
+      </c>
+      <c r="M21" t="str">
+        <f t="shared" si="2"/>
+        <v>OTHER DEPT</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
used not operator and learned ifna() and iferror() in error handling
</commit_message>
<xml_diff>
--- a/EXCEL/Details.xlsx
+++ b/EXCEL/Details.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/898af4500e89e0da/Desktop/DHRUV/Data Science and Analytics with GenAl/EXCEL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="28" documentId="8_{A6152608-415B-42DB-98F4-35F8CA028FB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D0E619BB-F5E3-44DD-9582-1116F9B9D094}"/>
+  <xr:revisionPtr revIDLastSave="29" documentId="8_{A6152608-415B-42DB-98F4-35F8CA028FB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EC4A3714-2603-4BDD-86D6-0A2725167AAA}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{5C010742-0D1E-4B81-84DF-4C0EBDAA81F1}"/>
   </bookViews>
@@ -568,6 +568,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CFD4C5C-D03E-4B7A-A44B-431478AFBB18}">
   <dimension ref="A1:M21"/>
   <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="13" max="13" width="10.640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A1" s="5" t="s">

</xml_diff>